<commit_message>
Update evaluation and attribute-assisted experiments
</commit_message>
<xml_diff>
--- a/data/labeled_data/1_FAIL/1_FAIL.xlsx
+++ b/data/labeled_data/1_FAIL/1_FAIL.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前50条视频审核" sheetId="1" r:id="R1e0a5e43b6cf4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前50条视频审核" sheetId="1" r:id="R4543d8ed67b34af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色编码规则" sheetId="2" r:id="Rdd25f3a135374c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="形状编码规则" sheetId="3" r:id="Rb303b79e4aad4925"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,12 +15,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="176" formatCode="0.0&quot; 秒（约）&quot;"/>
+    <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="23">
     <x:font>
@@ -590,7 +593,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -612,6 +615,28 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="50">
@@ -1061,6 +1086,12 @@
     <x:col min="5" max="5" width="27.77941131591797" customWidth="1"/>
     <x:col min="6" max="6" width="20" customWidth="1"/>
     <x:col min="7" max="7" width="17.77941131591797" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1085,9 +1116,25 @@
       <x:c r="G1" s="2" t="str">
         <x:v>reappearance_time</x:v>
       </x:c>
-      <x:c r="H1"/>
-      <x:c r="I1" s="6"/>
+      <x:c r="H1" s="8" t="str">
+        <x:v>清晰度评分（1–5）</x:v>
+      </x:c>
+      <x:c r="I1" s="9" t="str">
+        <x:v>流畅度评分（1–5）</x:v>
+      </x:c>
       <x:c r="J1" s="6"/>
+      <x:c r="K1" t="str">
+        <x:v>before_color</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>after_color</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>before_shape</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>after_shape</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -1111,9 +1158,25 @@
       <x:c r="G2" s="5" t="n">
         <x:v>2.6</x:v>
       </x:c>
-      <x:c r="H2"/>
-      <x:c r="I2" s="7"/>
+      <x:c r="H2" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I2" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J2" s="4"/>
+      <x:c r="K2" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="L2" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="M2" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="3" t="str">
@@ -1137,9 +1200,25 @@
       <x:c r="G3" s="5" t="n">
         <x:v>2.9</x:v>
       </x:c>
-      <x:c r="H3"/>
-      <x:c r="I3" s="7"/>
+      <x:c r="H3" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I3" s="13" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J3" s="4"/>
+      <x:c r="K3" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="L3" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="M3" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="N3" t="n">
+        <x:v>31</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="3" t="str">
@@ -1163,9 +1242,25 @@
       <x:c r="G4" s="5" t="n">
         <x:v>1.9</x:v>
       </x:c>
-      <x:c r="H4"/>
-      <x:c r="I4" s="7"/>
+      <x:c r="H4" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J4" s="4"/>
+      <x:c r="K4" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L4" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M4" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N4" t="n">
+        <x:v>43</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="3" t="str">
@@ -1189,9 +1284,25 @@
       <x:c r="G5" s="5" t="n">
         <x:v>2.6</x:v>
       </x:c>
-      <x:c r="H5"/>
-      <x:c r="I5" s="7"/>
+      <x:c r="H5" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I5" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J5" s="4"/>
+      <x:c r="K5" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L5" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M5" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N5" t="n">
+        <x:v>42</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="3" t="str">
@@ -1215,9 +1326,25 @@
       <x:c r="G6" s="5" t="n">
         <x:v>2.8</x:v>
       </x:c>
-      <x:c r="H6"/>
-      <x:c r="I6" s="7"/>
+      <x:c r="H6" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J6" s="4"/>
+      <x:c r="K6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M6" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N6" t="n">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="3" t="str">
@@ -1241,9 +1368,25 @@
       <x:c r="G7" s="5" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="H7"/>
-      <x:c r="I7" s="7"/>
+      <x:c r="H7" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I7" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J7" s="4"/>
+      <x:c r="K7" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L7" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M7" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N7" t="n">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="3" t="str">
@@ -1267,9 +1410,25 @@
       <x:c r="G8" s="5" t="n">
         <x:v>2.9</x:v>
       </x:c>
-      <x:c r="H8"/>
-      <x:c r="I8" s="7"/>
+      <x:c r="H8" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I8" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J8" s="4"/>
+      <x:c r="K8" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L8" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M8" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="N8" t="n">
+        <x:v>31</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="3" t="str">
@@ -1293,9 +1452,25 @@
       <x:c r="G9" s="5" t="n">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="H9"/>
-      <x:c r="I9" s="7"/>
+      <x:c r="H9" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I9" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J9" s="4"/>
+      <x:c r="K9" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="L9" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="M9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N9" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="3" t="str">
@@ -1319,9 +1494,25 @@
       <x:c r="G10" s="5" t="n">
         <x:v>2.5</x:v>
       </x:c>
-      <x:c r="H10"/>
-      <x:c r="I10" s="7"/>
+      <x:c r="H10" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I10" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J10" s="7"/>
+      <x:c r="K10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L10" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="M10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N10" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="3" t="str">
@@ -1345,9 +1536,25 @@
       <x:c r="G11" s="5" t="n">
         <x:v>2.7</x:v>
       </x:c>
-      <x:c r="H11"/>
-      <x:c r="I11" s="7"/>
+      <x:c r="H11" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I11" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J11" s="7"/>
+      <x:c r="K11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L11" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="M11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N11" t="n">
+        <x:v>32</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -1371,9 +1578,25 @@
       <x:c r="G12" s="5" t="n">
         <x:v>2.9</x:v>
       </x:c>
-      <x:c r="H12"/>
-      <x:c r="I12" s="7"/>
+      <x:c r="H12" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I12" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J12" s="7"/>
+      <x:c r="K12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N12" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="3" t="str">
@@ -1397,9 +1620,25 @@
       <x:c r="G13" s="5" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H13"/>
-      <x:c r="I13" s="7"/>
+      <x:c r="H13" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I13" s="13" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J13" s="7"/>
+      <x:c r="K13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L13" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="M13" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N13" t="n">
+        <x:v>78</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="3" t="str">
@@ -1423,9 +1662,25 @@
       <x:c r="G14" s="5" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H14"/>
-      <x:c r="I14"/>
+      <x:c r="H14" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I14" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J14"/>
+      <x:c r="K14" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L14" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M14" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N14" t="n">
+        <x:v>54</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="3" t="str">
@@ -1449,9 +1704,25 @@
       <x:c r="G15" s="5" t="n">
         <x:v>1.3</x:v>
       </x:c>
-      <x:c r="H15"/>
-      <x:c r="I15"/>
+      <x:c r="H15" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I15" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J15"/>
+      <x:c r="K15" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L15" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M15" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N15" t="n">
+        <x:v>56</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="3" t="str">
@@ -1475,9 +1746,25 @@
       <x:c r="G16" s="5" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="H16"/>
-      <x:c r="I16"/>
+      <x:c r="H16" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I16" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J16"/>
+      <x:c r="K16" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L16" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M16" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N16" t="n">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="3" t="str">
@@ -1501,9 +1788,25 @@
       <x:c r="G17" s="5" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17"/>
-      <x:c r="I17"/>
+      <x:c r="H17" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I17" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J17"/>
+      <x:c r="K17" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="L17" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M17" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N17" t="n">
+        <x:v>84</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="3" t="str">
@@ -1527,9 +1830,25 @@
       <x:c r="G18" s="5" t="n">
         <x:v>1.3</x:v>
       </x:c>
-      <x:c r="H18"/>
-      <x:c r="I18"/>
+      <x:c r="H18" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I18" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J18"/>
+      <x:c r="K18" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="L18" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M18" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N18" t="n">
+        <x:v>30</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="3" t="str">
@@ -1553,9 +1872,25 @@
       <x:c r="G19" s="5" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="H19"/>
-      <x:c r="I19"/>
+      <x:c r="H19" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I19" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J19"/>
+      <x:c r="K19" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="L19" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M19" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="N19" t="n">
+        <x:v>78</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
       <x:c r="A20" s="3" t="str">
@@ -1579,9 +1914,25 @@
       <x:c r="G20" s="5" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H20"/>
-      <x:c r="I20"/>
+      <x:c r="H20" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I20" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J20"/>
+      <x:c r="K20" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="L20" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="M20" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="N20" t="n">
+        <x:v>35</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="3" t="str">
@@ -1605,9 +1956,25 @@
       <x:c r="G21" s="5" t="n">
         <x:v>2.3</x:v>
       </x:c>
-      <x:c r="H21"/>
-      <x:c r="I21"/>
+      <x:c r="H21" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I21" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J21"/>
+      <x:c r="K21" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="L21" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M21" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="N21" t="n">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
       <x:c r="A22" s="3" t="str">
@@ -1631,9 +1998,25 @@
       <x:c r="G22" s="5" t="n">
         <x:v>1.8</x:v>
       </x:c>
-      <x:c r="H22"/>
-      <x:c r="I22"/>
+      <x:c r="H22" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I22" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J22"/>
+      <x:c r="K22" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L22" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="M22" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="N22" t="n">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
       <x:c r="A23" s="3" t="str">
@@ -1657,9 +2040,25 @@
       <x:c r="G23" s="5" t="n">
         <x:v>3.2</x:v>
       </x:c>
-      <x:c r="H23"/>
-      <x:c r="I23"/>
+      <x:c r="H23" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I23" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J23"/>
+      <x:c r="K23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M23" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="N23" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
       <x:c r="A24" s="3" t="str">
@@ -1683,9 +2082,25 @@
       <x:c r="G24" s="5" t="n">
         <x:v>1.2</x:v>
       </x:c>
-      <x:c r="H24"/>
-      <x:c r="I24"/>
+      <x:c r="H24" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I24" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J24"/>
+      <x:c r="K24" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="L24" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="M24" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N24" t="n">
+        <x:v>39</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="64" customHeight="1">
       <x:c r="A25" s="3" t="str">
@@ -1709,9 +2124,25 @@
       <x:c r="G25" s="5" t="n">
         <x:v>2.8</x:v>
       </x:c>
-      <x:c r="H25"/>
-      <x:c r="I25"/>
+      <x:c r="H25" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I25" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J25"/>
+      <x:c r="K25" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L25" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M25" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N25" t="n">
+        <x:v>28</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="64" customHeight="1">
       <x:c r="A26" s="3" t="str">
@@ -1735,9 +2166,25 @@
       <x:c r="G26" s="5" t="n">
         <x:v>3.1</x:v>
       </x:c>
-      <x:c r="H26"/>
-      <x:c r="I26"/>
+      <x:c r="H26" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I26" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J26"/>
+      <x:c r="K26" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L26" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="M26" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N26" t="n">
+        <x:v>79</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="64" customHeight="1">
       <x:c r="A27" s="3" t="str">
@@ -1761,9 +2208,25 @@
       <x:c r="G27" s="5" t="n">
         <x:v>3.7</x:v>
       </x:c>
-      <x:c r="H27"/>
-      <x:c r="I27"/>
+      <x:c r="H27" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I27" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J27"/>
+      <x:c r="K27" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L27" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="M27" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N27" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="64" customHeight="1">
       <x:c r="A28" s="3" t="str">
@@ -1787,9 +2250,25 @@
       <x:c r="G28" s="5" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H28"/>
-      <x:c r="I28"/>
+      <x:c r="H28" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I28" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J28"/>
+      <x:c r="K28" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="L28" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="M28" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N28" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="64" customHeight="1">
       <x:c r="A29" s="3" t="str">
@@ -1813,9 +2292,25 @@
       <x:c r="G29" s="5" t="n">
         <x:v>3.1</x:v>
       </x:c>
-      <x:c r="H29"/>
-      <x:c r="I29"/>
+      <x:c r="H29" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I29" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J29"/>
+      <x:c r="K29" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="L29" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="M29" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="N29" t="n">
+        <x:v>76</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="64" customHeight="1">
       <x:c r="A30" s="3" t="str">
@@ -1839,9 +2334,25 @@
       <x:c r="G30" s="5" t="n">
         <x:v>2.8</x:v>
       </x:c>
-      <x:c r="H30"/>
-      <x:c r="I30"/>
+      <x:c r="H30" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I30" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J30"/>
+      <x:c r="K30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N30" t="n">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="64" customHeight="1">
       <x:c r="A31" s="3" t="str">
@@ -1865,9 +2376,25 @@
       <x:c r="G31" s="5" t="n">
         <x:v>2.6</x:v>
       </x:c>
-      <x:c r="H31"/>
-      <x:c r="I31"/>
+      <x:c r="H31" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I31" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J31"/>
+      <x:c r="K31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M31" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N31" t="n">
+        <x:v>19</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="64" customHeight="1">
       <x:c r="A32" s="3" t="str">
@@ -1891,9 +2418,25 @@
       <x:c r="G32" s="5" t="n">
         <x:v>1.6</x:v>
       </x:c>
-      <x:c r="H32"/>
-      <x:c r="I32"/>
+      <x:c r="H32" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I32" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J32"/>
+      <x:c r="K32" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="L32" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="M32" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N32" t="n">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="64" customHeight="1">
       <x:c r="A33" s="3" t="str">
@@ -1917,9 +2460,25 @@
       <x:c r="G33" s="5" t="n">
         <x:v>2.8</x:v>
       </x:c>
-      <x:c r="H33"/>
-      <x:c r="I33"/>
+      <x:c r="H33" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I33" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J33"/>
+      <x:c r="K33" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="L33" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="M33" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N33" t="n">
+        <x:v>11</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="64" customHeight="1">
       <x:c r="A34" s="3" t="str">
@@ -1943,9 +2502,25 @@
       <x:c r="G34" s="5" t="n">
         <x:v>1.4</x:v>
       </x:c>
-      <x:c r="H34"/>
-      <x:c r="I34"/>
+      <x:c r="H34" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I34" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J34"/>
+      <x:c r="K34" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L34" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M34" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N34" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="64" customHeight="1">
       <x:c r="A35" s="3" t="str">
@@ -1969,9 +2544,25 @@
       <x:c r="G35" s="5" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H35"/>
-      <x:c r="I35"/>
+      <x:c r="H35" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I35" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J35"/>
+      <x:c r="K35" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L35" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M35" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N35" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="64" customHeight="1">
       <x:c r="A36" s="3" t="str">
@@ -1995,9 +2586,25 @@
       <x:c r="G36" s="5" t="n">
         <x:v>0.4</x:v>
       </x:c>
-      <x:c r="H36"/>
-      <x:c r="I36"/>
+      <x:c r="H36" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I36" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J36"/>
+      <x:c r="K36" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L36" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M36" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N36" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="64" customHeight="1">
       <x:c r="A37" s="3" t="str">
@@ -2021,9 +2628,25 @@
       <x:c r="G37" s="5" t="n">
         <x:v>2.6</x:v>
       </x:c>
-      <x:c r="H37"/>
-      <x:c r="I37"/>
+      <x:c r="H37" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I37" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J37"/>
+      <x:c r="K37" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L37" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="M37" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N37" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="64" customHeight="1">
       <x:c r="A38" s="3" t="str">
@@ -2047,9 +2670,25 @@
       <x:c r="G38" s="5" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="H38"/>
-      <x:c r="I38"/>
+      <x:c r="H38" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I38" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J38"/>
+      <x:c r="K38" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L38" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="M38" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N38" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="64" customHeight="1">
       <x:c r="A39" s="3" t="str">
@@ -2073,9 +2712,25 @@
       <x:c r="G39" s="5" t="n">
         <x:v>1.7</x:v>
       </x:c>
-      <x:c r="H39"/>
-      <x:c r="I39"/>
+      <x:c r="H39" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I39" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J39"/>
+      <x:c r="K39" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L39" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M39" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N39" t="n">
+        <x:v>84</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="64" customHeight="1">
       <x:c r="A40" s="3" t="str">
@@ -2099,9 +2754,25 @@
       <x:c r="G40" s="5" t="n">
         <x:v>1.7</x:v>
       </x:c>
-      <x:c r="H40"/>
-      <x:c r="I40"/>
+      <x:c r="H40" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I40" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J40"/>
+      <x:c r="K40" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L40" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M40" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N40" t="n">
+        <x:v>84</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="64" customHeight="1">
       <x:c r="A41" s="3" t="str">
@@ -2125,9 +2796,25 @@
       <x:c r="G41" s="5" t="n">
         <x:v>1.9</x:v>
       </x:c>
-      <x:c r="H41"/>
-      <x:c r="I41"/>
+      <x:c r="H41" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I41" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J41"/>
+      <x:c r="K41" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L41" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M41" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="N41" t="n">
+        <x:v>68</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="64" customHeight="1">
       <x:c r="A42" s="3" t="str">
@@ -2151,152 +2838,248 @@
       <x:c r="G42" s="5" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H42"/>
-      <x:c r="I42"/>
+      <x:c r="H42" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I42" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="J42"/>
+      <x:c r="K42" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L42" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="M42" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="N42" t="n">
+        <x:v>40</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="64" customHeight="1">
       <x:c r="A43" s="3" t="str">
-        <x:v>C0409</x:v>
+        <x:v>C0455</x:v>
       </x:c>
       <x:c r="B43" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C43" s="4" t="str">
-        <x:v>后段挡板扭曲、移开并露出原目标区域，球体却不见，出现目标消失异常。</x:v>
+        <x:v>补帧确认重现后的金色球体新增明显纵向深色条纹和网格纹理，表面外观与遮挡前不一致。</x:v>
       </x:c>
       <x:c r="D43" s="4" t="str">
-        <x:v>青蓝色→未见</x:v>
+        <x:v>紫色、金黄色→紫色、金黄色</x:v>
       </x:c>
       <x:c r="E43" s="4" t="str">
-        <x:v>球形→消失</x:v>
+        <x:v>方块、光滑球体→方块、带纵向条纹的球体</x:v>
       </x:c>
       <x:c r="F43" s="5" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="G43" s="5" t="str">
-        <x:v>未重现</x:v>
-      </x:c>
-      <x:c r="H43"/>
-      <x:c r="I43"/>
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="G43" s="5" t="n">
+        <x:v>3.1</x:v>
+      </x:c>
+      <x:c r="H43" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I43" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J43"/>
+      <x:c r="K43" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="L43" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="M43" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="N43" t="n">
+        <x:v>63</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="64" customHeight="1">
       <x:c r="A44" s="3" t="str">
-        <x:v>C0455</x:v>
+        <x:v>C0483</x:v>
       </x:c>
       <x:c r="B44" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C44" s="4" t="str">
-        <x:v>补帧确认重现后的金色球体新增明显纵向深色条纹和网格纹理，表面外观与遮挡前不一致。</x:v>
+        <x:v>遮挡前为绿色球体，挡板升起后重现为红色，颜色明显改变。</x:v>
       </x:c>
       <x:c r="D44" s="4" t="str">
-        <x:v>紫色、金黄色→紫色、金黄色</x:v>
+        <x:v>绿色→红色</x:v>
       </x:c>
       <x:c r="E44" s="4" t="str">
-        <x:v>方块、光滑球体→方块、带纵向条纹的球体</x:v>
+        <x:v>球形→球形</x:v>
       </x:c>
       <x:c r="F44" s="5" t="n">
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="G44" s="5" t="n">
-        <x:v>3.1</x:v>
-      </x:c>
-      <x:c r="H44"/>
-      <x:c r="I44"/>
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="H44" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I44" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="J44"/>
+      <x:c r="K44" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L44" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M44" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="N44" t="n">
+        <x:v>76</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="64" customHeight="1">
       <x:c r="A45" s="3" t="str">
-        <x:v>C0483</x:v>
+        <x:v>C0493</x:v>
       </x:c>
       <x:c r="B45" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C45" s="4" t="str">
-        <x:v>遮挡前为绿色球体，挡板升起后重现为红色，颜色明显改变。</x:v>
+        <x:v>原青蓝球体被遮住后，约2.8秒左侧新增灰白球体；随后青蓝球体在右侧重现，目标数量及出现过程异常。</x:v>
       </x:c>
       <x:c r="D45" s="4" t="str">
-        <x:v>绿色→红色</x:v>
+        <x:v>青蓝色→青蓝色及灰白色</x:v>
       </x:c>
       <x:c r="E45" s="4" t="str">
-        <x:v>球形→球形</x:v>
+        <x:v>单个球体→新增灰白球体</x:v>
       </x:c>
       <x:c r="F45" s="5" t="n">
-        <x:v>1.9</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="G45" s="5" t="n">
-        <x:v>3.7</x:v>
-      </x:c>
-      <x:c r="H45"/>
-      <x:c r="I45"/>
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="H45" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I45" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="J45"/>
+      <x:c r="K45" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L45" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="M45" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="N45" t="n">
+        <x:v>58</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="64" customHeight="1">
       <x:c r="A46" s="3" t="str">
-        <x:v>C0493</x:v>
+        <x:v>C0497</x:v>
       </x:c>
       <x:c r="B46" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C46" s="4" t="str">
-        <x:v>原青蓝球体被遮住后，约2.8秒左侧新增灰白球体；随后青蓝球体在右侧重现，目标数量及出现过程异常。</x:v>
+        <x:v>遮挡前为青蓝色球体，右侧重现后变为红色，颜色明显改变。</x:v>
       </x:c>
       <x:c r="D46" s="4" t="str">
-        <x:v>青蓝色→青蓝色及灰白色</x:v>
+        <x:v>青蓝色→红色</x:v>
       </x:c>
       <x:c r="E46" s="4" t="str">
-        <x:v>单个球体→新增灰白球体</x:v>
+        <x:v>球形→球形</x:v>
       </x:c>
       <x:c r="F46" s="5" t="n">
-        <x:v>1.2</x:v>
+        <x:v>1.9</x:v>
       </x:c>
       <x:c r="G46" s="5" t="n">
-        <x:v>2.8</x:v>
-      </x:c>
-      <x:c r="H46"/>
-      <x:c r="I46"/>
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="H46" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I46" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="J46"/>
+      <x:c r="K46" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M46" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="N46" t="n">
+        <x:v>76</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="64" customHeight="1">
       <x:c r="A47" s="3" t="str">
-        <x:v>C0497</x:v>
+        <x:v>C0507</x:v>
       </x:c>
       <x:c r="B47" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C47" s="4" t="str">
-        <x:v>遮挡前为青蓝色球体，右侧重现后变为红色，颜色明显改变。</x:v>
+        <x:v>挡板下降后左侧方块由绿色变红色，右侧由紫色变蓝色，颜色明显改变。</x:v>
       </x:c>
       <x:c r="D47" s="4" t="str">
-        <x:v>青蓝色→红色</x:v>
+        <x:v>绿色、紫色→红色、蓝色</x:v>
       </x:c>
       <x:c r="E47" s="4" t="str">
-        <x:v>球形→球形</x:v>
+        <x:v>两个方块→两个方块</x:v>
       </x:c>
       <x:c r="F47" s="5" t="n">
-        <x:v>1.9</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="G47" s="5" t="n">
-        <x:v>4.3</x:v>
-      </x:c>
-      <x:c r="H47"/>
-      <x:c r="I47"/>
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="H47" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="J47"/>
+      <x:c r="K47" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="L47" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="M47" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N47" t="n">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="64" customHeight="1">
       <x:c r="A48" s="3" t="str">
-        <x:v>C0507</x:v>
+        <x:v>C0521</x:v>
       </x:c>
       <x:c r="B48" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C48" s="4" t="str">
-        <x:v>挡板下降后左侧方块由绿色变红色，右侧由紫色变蓝色，颜色明显改变。</x:v>
+        <x:v>重现后左侧方块由绿色变蓝色，右侧由青蓝色变红色，颜色明显改变。</x:v>
       </x:c>
       <x:c r="D48" s="4" t="str">
-        <x:v>绿色、紫色→红色、蓝色</x:v>
+        <x:v>绿色、青蓝色→蓝色、红色</x:v>
       </x:c>
       <x:c r="E48" s="4" t="str">
         <x:v>两个方块→两个方块</x:v>
@@ -2307,35 +3090,41 @@
       <x:c r="G48" s="5" t="n">
         <x:v>4.5</x:v>
       </x:c>
-      <x:c r="H48"/>
-      <x:c r="I48"/>
+      <x:c r="H48" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="J48"/>
+      <x:c r="K48" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="L48" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="M48" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N48" t="n">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="64" customHeight="1">
-      <x:c r="A49" s="3" t="str">
-        <x:v>C0521</x:v>
-      </x:c>
-      <x:c r="B49" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C49" s="4" t="str">
-        <x:v>重现后左侧方块由绿色变蓝色，右侧由青蓝色变红色，颜色明显改变。</x:v>
-      </x:c>
-      <x:c r="D49" s="4" t="str">
-        <x:v>绿色、青蓝色→蓝色、红色</x:v>
-      </x:c>
-      <x:c r="E49" s="4" t="str">
-        <x:v>两个方块→两个方块</x:v>
-      </x:c>
-      <x:c r="F49" s="5" t="n">
-        <x:v>1.2</x:v>
-      </x:c>
-      <x:c r="G49" s="5" t="n">
-        <x:v>4.5</x:v>
-      </x:c>
+      <x:c r="A49" s="3"/>
+      <x:c r="B49" s="3"/>
+      <x:c r="C49" s="4"/>
+      <x:c r="D49" s="4"/>
+      <x:c r="E49" s="4"/>
+      <x:c r="F49" s="5"/>
+      <x:c r="G49" s="5"/>
       <x:c r="H49"/>
       <x:c r="I49"/>
       <x:c r="J49"/>
+      <x:c r="K49"/>
+      <x:c r="L49"/>
+      <x:c r="M49"/>
+      <x:c r="N49"/>
     </x:row>
     <x:row r="50" ht="64" customHeight="1">
       <x:c r="A50" s="3"/>
@@ -2345,6 +3134,10 @@
       <x:c r="E50" s="4"/>
       <x:c r="F50" s="5"/>
       <x:c r="G50" s="5"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
+      <x:c r="N50"/>
     </x:row>
     <x:row r="51" ht="64" customHeight="1">
       <x:c r="A51" s="3"/>
@@ -2354,6 +3147,10 @@
       <x:c r="E51" s="4"/>
       <x:c r="F51" s="5"/>
       <x:c r="G51" s="5"/>
+      <x:c r="K51"/>
+      <x:c r="L51"/>
+      <x:c r="M51"/>
+      <x:c r="N51"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B2:B51">
@@ -2361,6 +3158,1784 @@
       <x:formula>1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="whole" operator="between" sqref="H2:I48">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="82" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" t="str">
+        <x:v>颜色编码</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>颜色名称或状态</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>规则</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>红色</x:v>
+      </x:c>
+      <x:c r="D2" s="15" t="str">
+        <x:v>正整数</x:v>
+      </x:c>
+      <x:c r="E2" s="15" t="str">
+        <x:v>颜色或完整多色组合的类别编号；不能按数值大小或相减解释色差。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="44" customHeight="1">
+      <x:c r="A3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>蓝色</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="str">
+        <x:v>红/蓝</x:v>
+      </x:c>
+      <x:c r="E3" s="15" t="str">
+        <x:v>红色=1；蓝色=2；所有Excel共用同一套编码。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="44" customHeight="1">
+      <x:c r="A4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>绿色</x:v>
+      </x:c>
+      <x:c r="D4" s="15" t="str">
+        <x:v>色调保留</x:v>
+      </x:c>
+      <x:c r="E4" s="15" t="str">
+        <x:v>浅、深、亮、灰等明确色调和多色组合保持独立类别；不自动合并。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>黄色</x:v>
+      </x:c>
+      <x:c r="D5" s="15" t="str">
+        <x:v>方向</x:v>
+      </x:c>
+      <x:c r="E5" s="15" t="str">
+        <x:v>以→拆分；before取第一段，after取最后一段；中间过程保留在原color列。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>橙色</x:v>
+      </x:c>
+      <x:c r="D6" s="15" t="str">
+        <x:v>括号</x:v>
+      </x:c>
+      <x:c r="E6" s="15" t="str">
+        <x:v>移除局部、淡化、半透明等括号说明，原color列保留完整文字。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>紫色</x:v>
+      </x:c>
+      <x:c r="D7" s="15" t="str">
+        <x:v>全程</x:v>
+      </x:c>
+      <x:c r="E7" s="15" t="str">
+        <x:v>标为全程且有明确颜色时，将相同编码填入前后两列；不代表遮挡事件有效。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>粉色</x:v>
+      </x:c>
+      <x:c r="D8" s="15" t="str">
+        <x:v>无前后对照</x:v>
+      </x:c>
+      <x:c r="E8" s="15" t="str">
+        <x:v>明确未形成有效前后对照，或无箭头且无全程说明时，两列为-5。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>棕色</x:v>
+      </x:c>
+      <x:c r="D9" s="15" t="str">
+        <x:v>缺失</x:v>
+      </x:c>
+      <x:c r="E9" s="15" t="str">
+        <x:v>实际视频缺少color时仅按同一ID查原始raw_data；仍缺失为-1；空白行不填。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="A10" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>黑色</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="str">
+        <x:v>多色</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="str">
+        <x:v>按完整文字组合编码；不推断不同物体对应关系，组合顺序不同也不强行等同。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="44" customHeight="1">
+      <x:c r="A11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>白色</x:v>
+      </x:c>
+      <x:c r="D11" s="15" t="str">
+        <x:v>保留</x:v>
+      </x:c>
+      <x:c r="E11" s="15" t="str">
+        <x:v>原color列、其他列、标签、顺序全部保留；新增两列及本编码表。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>金色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>银色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>亮粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>亮粉色、蓝色、浅绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>亮绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>亮绿色、蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>亮青色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>亮黄绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>土黄色、粉紫色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>棕橙色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>棕灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>棕色、红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>棕色、蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>棕金色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>棕黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>橄榄黄绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>橙红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>橙红色、浅棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>橙色、棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>橙金色发光</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>橙黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>浅棕色、红棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>浅粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>浅绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>浅蓝色、红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>浅青色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>浅青色、蓝色、浅青色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>浅黄绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>浅黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>淡红灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>深灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>深灰黑色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>深蓝灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>深蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>深青色、蓝色、粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>灰棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>灰白杂色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>灰白色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>灰粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>灰绿、棕色高光</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>灰绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>灰色、浅紫色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>灰色、淡紫色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>灰色、粉紫色、深绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>灰色、粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>灰色、青蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>灰蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>灰青色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>白色带彩色点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>米白色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>粉红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>紫红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>紫色、深绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>紫色、深蓝色、亮绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>紫色、深蓝色、浅绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>紫色、白色边缘</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>紫色、红色、深蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>紫色、红色、蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>紫色、蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>紫色、蓝色、浅绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>紫色、蓝色、绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>紫色、金黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>红棕色、青红双色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>红色、蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>绿色、紫色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>绿色、青蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>肤色及棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>蓝灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>蓝白色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>蓝色、棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>蓝色、红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>金色、棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>金黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>银灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>青绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>青绿色、橙色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>青绿色、灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>青绿色、灰蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>青色、深蓝色、亮粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>青色、蓝色、粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>青蓝色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>青蓝色、橙红色等</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>青蓝色、深蓝色、粉色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>青蓝色、灰白色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>青蓝色、灰色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>青蓝色、灰色不明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>青蓝色及灰白色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>黄橙色、棕色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>黄绿色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>黄色、蓝色、橙红色、黄色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>黄色带深色斑块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>黑白反光色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>黑红交替</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>黑色、白色底座</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>黑褐色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>无法辨认或缺少颜色记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="n">
+        <x:v>-2</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>未见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="n">
+        <x:v>-3</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>未重现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="n">
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>消失或逐渐消失</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="n">
+        <x:v>-5</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>缺少可明确分配的前后对照</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="82" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" t="str">
+        <x:v>形状编码</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>形状描述或状态</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>规则</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>球体</x:v>
+      </x:c>
+      <x:c r="D2" s="15" t="str">
+        <x:v>类别编号</x:v>
+      </x:c>
+      <x:c r="E2" s="15" t="str">
+        <x:v>正整数是形状描述的类别编号，不表示大小、差异程度或评分。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="44" customHeight="1">
+      <x:c r="A3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>立方体</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="str">
+        <x:v>基本形状</x:v>
+      </x:c>
+      <x:c r="E3" s="15" t="str">
+        <x:v>球体=1；立方体=2；圆柱体=3；棱锥=4；圆盘形=5。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="44" customHeight="1">
+      <x:c r="A4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>圆柱体</x:v>
+      </x:c>
+      <x:c r="D4" s="15" t="str">
+        <x:v>描述保留</x:v>
+      </x:c>
+      <x:c r="E4" s="15" t="str">
+        <x:v>不同措辞、大小、数量、局部可见、纹理与形变描述保持独立类别；不自动合并同义词。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>棱锥</x:v>
+      </x:c>
+      <x:c r="D5" s="15" t="str">
+        <x:v>方向</x:v>
+      </x:c>
+      <x:c r="E5" s="15" t="str">
+        <x:v>按→拆分，before取第一段、after取最后一段；中间状态仍在原shape列中。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>圆盘形</x:v>
+      </x:c>
+      <x:c r="D6" s="15" t="str">
+        <x:v>括号</x:v>
+      </x:c>
+      <x:c r="E6" s="15" t="str">
+        <x:v>仅移除全程说明；短暂双球、后恢复一个等括号信息保留并独立编码。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>一个圆盘</x:v>
+      </x:c>
+      <x:c r="D7" s="15" t="str">
+        <x:v>全程</x:v>
+      </x:c>
+      <x:c r="E7" s="15" t="str">
+        <x:v>原记录明确全程时，前后填相同编号；不表示遮挡事件有效。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>一个球体</x:v>
+      </x:c>
+      <x:c r="D8" s="15" t="str">
+        <x:v>无明确前后</x:v>
+      </x:c>
+      <x:c r="E8" s="15" t="str">
+        <x:v>无箭头且无全程说明时，前后均为-5，不猜测前后形状。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>一个近球形目标</x:v>
+      </x:c>
+      <x:c r="D9" s="15" t="str">
+        <x:v>缺失</x:v>
+      </x:c>
+      <x:c r="E9" s="15" t="str">
+        <x:v>shape为空时按同一ID查询raw_data；仍无信息则为-1；空白行不填。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="A10" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>上部圆顶、下部方形</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="str">
+        <x:v>保留</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="str">
+        <x:v>原shape、color、颜色编码、评分、标签及现有编码表均不修改。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>不稳定的扁圆团块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>不规则团状</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>不规则近球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>两个圆盘</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>两个小球体（后恢复一个）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>两个带底座的柱状物</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>两个方块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>两个棱锥和一个方块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>两个球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>两个目标局部同时可见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>两侧同时出现球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>人头状物体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>仅一个球体可追踪</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>仅局部可见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>仅方块重现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>仅见上部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>仅见部分圆弧</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>仅青蓝色球可辨认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>先后出现三个球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>光滑小球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>凹凸不规则摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>凹凸不规则近球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>半透明局部球影</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>单个球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>变大球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>变大球形摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>四个方块的下部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>圆形主体带底座</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>圆盘状摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>多个不规则球影</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>多个重叠或变形球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>大球体、圆柱体、小球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>小球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>小球体（短暂双球）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>小球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>小球形摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>局部可见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>局部圆形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>局部球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>局部被遮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>带小孔的两个方块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>带小突起的球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>带环状细线的球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>带纵纹球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>扁化不规则摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>扁化摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>扁圆不规则摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>扁多面体、圆柱体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>新增灰白球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>方块、光滑球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>方块、圆柱体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>方块、带把手杯状物</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>方块、带环纹球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>方块、带纵向条纹的球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>方块、球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>方块、较高长方体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>方块形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>方块被遮住、球体异常显现在挡板表面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>明显变大的球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>棱锥形局部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>模糊后重现球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>模糊团块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>水滴状不规则团块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>球体、方块</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>球体、方块、棱锥</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>球体及尖顶物体局部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>球形局部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>球形摆锤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>至少三个球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>较大球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>近球形</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>部分球体</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>部分露出</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>重复球影</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>无法辨认或缺少形状记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="n">
+        <x:v>-2</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>未见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="n">
+        <x:v>-3</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>未重现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="n">
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>消失或逐渐消失</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="n">
+        <x:v>-5</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>缺少可明确分配的前后对照</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>